<commit_message>
Make comp plans and ISPs data-driven from the sheet
- Sheet gains CompPlans (seeded from Sequifi export) and ISPs tabs.
- doGet returns roster + compPlans + isps in one bootstrap call.
- Form: comp is now a dropdown of named plans pulled from CompPlans;
  ISP chips pulled from ISPs; picking a rep prefills their default plan.
- New ISPs submitted on the form append back to the ISPs tab.
- Roster now carries "Default plan"; template seeds plans per rep.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/Unbreakable-Blitz-Intake-Template.xlsx
+++ b/template/Unbreakable-Blitz-Intake-Template.xlsx
@@ -9,7 +9,9 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Roster" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Submissions" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="CompPlans" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="ISPs" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Submissions" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="9">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -61,12 +63,6 @@
       <name val="Arial"/>
       <b val="1"/>
       <color rgb="003A2A00"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <b val="1"/>
-      <color rgb="00FFFFFF"/>
-      <sz val="11"/>
     </font>
     <font>
       <name val="Arial"/>
@@ -123,7 +119,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -131,17 +127,14 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -507,11 +500,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B22"/>
+  <dimension ref="B2:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
-    <col width="100" customWidth="1" min="2" max="2"/>
+    <col width="104" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="2">
@@ -524,93 +517,84 @@
     <row r="3">
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>This one Google Sheet is the datastore for the blitz intake form. Two tabs do the work.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="B4" t="inlineStr"/>
+          <t>One Google Sheet powers the intake form. The form pulls its dropdowns from the reference tabs below.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
-          <t>What your CS team fills in</t>
+          <t>Tabs the form PULLS FROM (edit these to change the form's options)</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• The Roster tab — the master rep list. Complete the yellow columns (Email, Default comp) and add any missing reps.</t>
+          <t>• Roster — master rep list. The form's rep picker reads this. Fill the yellow Email column; verify Default plan.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>• Region is set from the UNB ID prefix (1xxx=NY, 2xxx=MA, 3xxx=AL, 4xxx=CT, 5xxx=ME, 6xxx/9xxx=Call Center).</t>
+          <t>• CompPlans — Sequifi's named rate plans. The form's comp dropdown reads this. Add a row to add a plan.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>• Default comp is optional — it just pre-fills the form. Actual comp is set per blitz on the form itself.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" t="inlineStr"/>
+          <t>• ISPs — the ISP chips on the form read this. Add a row (name + abbr) to add a selectable ISP.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>What fills in automatically</t>
+          <t>Tab that FILLS AUTOMATICALLY</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="B11" s="4" t="inlineStr">
         <is>
-          <t>• The Submissions tab — one row per blitz submitted through the form. Do not edit its header row.</t>
+          <t>• Submissions — one row per blitz submitted. New reps + new ISPs from the form append back to Roster / ISPs.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>• New reps added on the form (first / last / email) are appended to the Roster tab automatically.</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" t="inlineStr"/>
+          <t>• Do not edit the Submissions header row.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>How to turn this sheet into the live backend (one-time, ~2 min)</t>
+          <t>Make it live (one-time, ~2 min)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" s="4" t="inlineStr">
         <is>
-          <t>1. File → Make sure this is a Google Sheet (if imported from .xlsx, it already is).</t>
+          <t>1. This file is already a Google Sheet once imported to Drive.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>2. Extensions → Apps Script. Delete the sample, paste the Code.gs from the project, Save.</t>
+          <t>2. Extensions → Apps Script → paste Code.gs → Save.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="B17" s="4" t="inlineStr">
         <is>
-          <t>3. Deploy → New deployment → Web app. Execute as: Me. Who has access: Anyone. Deploy &amp; authorize.</t>
+          <t>3. Deploy → New deployment → Web app. Execute as: Me. Access: Anyone. Deploy &amp; authorize.</t>
         </is>
       </c>
     </row>
@@ -624,24 +608,14 @@
     <row r="19">
       <c r="B19" s="4" t="inlineStr">
         <is>
-          <t>5. Open the intake form → Connect → paste that URL.  (Form: https://unbreakable-blitz-intake.vercel.app)</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" t="inlineStr"/>
+          <t>5. Intake form → Connect → paste the URL.   Form: https://unbreakable-blitz-intake.vercel.app</t>
+        </is>
+      </c>
     </row>
     <row r="21">
-      <c r="B21" s="3" t="inlineStr">
-        <is>
-          <t>Legend</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="5" t="inlineStr">
-        <is>
-          <t>Yellow columns = fill these in.   White columns = leave as-is / auto-filled.</t>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Yellow columns = fill / verify these.   White = leave as-is or auto-filled.</t>
         </is>
       </c>
     </row>
@@ -663,11 +637,11 @@
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="20" customHeight="1">
+    <row r="1" ht="24" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
           <t>First</t>
@@ -690,7 +664,7 @@
       </c>
       <c r="E1" s="7" t="inlineStr">
         <is>
-          <t>Default comp</t>
+          <t>Default plan</t>
         </is>
       </c>
       <c r="F1" s="6" t="inlineStr">
@@ -716,7 +690,11 @@
           <t>UNB1001</t>
         </is>
       </c>
-      <c r="E2" s="9" t="inlineStr"/>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>Rate 325</t>
+        </is>
+      </c>
       <c r="F2" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -740,7 +718,11 @@
           <t>UNB1002</t>
         </is>
       </c>
-      <c r="E3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F3" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -764,7 +746,11 @@
           <t>UNB1003</t>
         </is>
       </c>
-      <c r="E4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F4" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -792,7 +778,11 @@
           <t>UNB1004</t>
         </is>
       </c>
-      <c r="E5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F5" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -816,7 +806,11 @@
           <t>UNB1005</t>
         </is>
       </c>
-      <c r="E6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F6" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -864,7 +858,11 @@
           <t>UNB1007</t>
         </is>
       </c>
-      <c r="E8" s="9" t="inlineStr"/>
+      <c r="E8" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F8" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -888,7 +886,11 @@
           <t>UNB1008</t>
         </is>
       </c>
-      <c r="E9" s="9" t="inlineStr"/>
+      <c r="E9" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F9" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -912,7 +914,11 @@
           <t>UNB1009</t>
         </is>
       </c>
-      <c r="E10" s="9" t="inlineStr"/>
+      <c r="E10" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F10" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -960,7 +966,11 @@
           <t>UNB1011</t>
         </is>
       </c>
-      <c r="E12" s="9" t="inlineStr"/>
+      <c r="E12" s="9" t="inlineStr">
+        <is>
+          <t>Rate 275</t>
+        </is>
+      </c>
       <c r="F12" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -988,7 +998,11 @@
           <t>UNB1012</t>
         </is>
       </c>
-      <c r="E13" s="9" t="inlineStr"/>
+      <c r="E13" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F13" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -1016,7 +1030,11 @@
           <t>UNB1013</t>
         </is>
       </c>
-      <c r="E14" s="9" t="inlineStr"/>
+      <c r="E14" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F14" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -1044,7 +1062,11 @@
           <t>UNB1014</t>
         </is>
       </c>
-      <c r="E15" s="9" t="inlineStr"/>
+      <c r="E15" s="9" t="inlineStr">
+        <is>
+          <t>Rate 200</t>
+        </is>
+      </c>
       <c r="F15" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -1092,7 +1114,11 @@
           <t>UNB1016</t>
         </is>
       </c>
-      <c r="E17" s="9" t="inlineStr"/>
+      <c r="E17" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F17" s="8" t="inlineStr">
         <is>
           <t>NY</t>
@@ -1164,7 +1190,11 @@
           <t>UNB2003</t>
         </is>
       </c>
-      <c r="E20" s="9" t="inlineStr"/>
+      <c r="E20" s="9" t="inlineStr">
+        <is>
+          <t>Rate 225</t>
+        </is>
+      </c>
       <c r="F20" s="8" t="inlineStr">
         <is>
           <t>MA</t>
@@ -1212,7 +1242,11 @@
           <t>UNB2005</t>
         </is>
       </c>
-      <c r="E22" s="9" t="inlineStr"/>
+      <c r="E22" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F22" s="8" t="inlineStr">
         <is>
           <t>MA</t>
@@ -1236,7 +1270,11 @@
           <t>UNB2006</t>
         </is>
       </c>
-      <c r="E23" s="9" t="inlineStr"/>
+      <c r="E23" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F23" s="8" t="inlineStr">
         <is>
           <t>MA</t>
@@ -1260,7 +1298,11 @@
           <t>UNB2007</t>
         </is>
       </c>
-      <c r="E24" s="9" t="inlineStr"/>
+      <c r="E24" s="9" t="inlineStr">
+        <is>
+          <t>Rate 200</t>
+        </is>
+      </c>
       <c r="F24" s="8" t="inlineStr">
         <is>
           <t>MA</t>
@@ -1424,7 +1466,11 @@
           <t>UNB3001</t>
         </is>
       </c>
-      <c r="E31" s="9" t="inlineStr"/>
+      <c r="E31" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F31" s="8" t="inlineStr">
         <is>
           <t>AL</t>
@@ -1544,7 +1590,11 @@
           <t>UNB3006</t>
         </is>
       </c>
-      <c r="E36" s="9" t="inlineStr"/>
+      <c r="E36" s="9" t="inlineStr">
+        <is>
+          <t>Rate 225</t>
+        </is>
+      </c>
       <c r="F36" s="8" t="inlineStr">
         <is>
           <t>AL</t>
@@ -1588,7 +1638,11 @@
           <t>UNB3008</t>
         </is>
       </c>
-      <c r="E38" s="9" t="inlineStr"/>
+      <c r="E38" s="9" t="inlineStr">
+        <is>
+          <t>Rate 300</t>
+        </is>
+      </c>
       <c r="F38" s="8" t="inlineStr">
         <is>
           <t>AL</t>
@@ -1612,7 +1666,11 @@
           <t>UNB3009</t>
         </is>
       </c>
-      <c r="E39" s="9" t="inlineStr"/>
+      <c r="E39" s="9" t="inlineStr">
+        <is>
+          <t>Rate 225</t>
+        </is>
+      </c>
       <c r="F39" s="8" t="inlineStr">
         <is>
           <t>AL</t>
@@ -1684,7 +1742,11 @@
           <t>UNB4003</t>
         </is>
       </c>
-      <c r="E42" s="9" t="inlineStr"/>
+      <c r="E42" s="9" t="inlineStr">
+        <is>
+          <t>Rate 325</t>
+        </is>
+      </c>
       <c r="F42" s="8" t="inlineStr">
         <is>
           <t>CT</t>
@@ -1708,7 +1770,11 @@
           <t>UNB4004</t>
         </is>
       </c>
-      <c r="E43" s="9" t="inlineStr"/>
+      <c r="E43" s="9" t="inlineStr">
+        <is>
+          <t>Rate 325</t>
+        </is>
+      </c>
       <c r="F43" s="8" t="inlineStr">
         <is>
           <t>CT</t>
@@ -1732,7 +1798,11 @@
           <t>UNB5001</t>
         </is>
       </c>
-      <c r="E44" s="9" t="inlineStr"/>
+      <c r="E44" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F44" s="8" t="inlineStr">
         <is>
           <t>ME</t>
@@ -1756,7 +1826,11 @@
           <t>UNB5002</t>
         </is>
       </c>
-      <c r="E45" s="9" t="inlineStr"/>
+      <c r="E45" s="9" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
       <c r="F45" s="8" t="inlineStr">
         <is>
           <t>ME</t>
@@ -1780,7 +1854,11 @@
           <t>UNB5003</t>
         </is>
       </c>
-      <c r="E46" s="9" t="inlineStr"/>
+      <c r="E46" s="9" t="inlineStr">
+        <is>
+          <t>Rate 200</t>
+        </is>
+      </c>
       <c r="F46" s="8" t="inlineStr">
         <is>
           <t>ME</t>
@@ -1804,7 +1882,11 @@
           <t>UNB5004</t>
         </is>
       </c>
-      <c r="E47" s="9" t="inlineStr"/>
+      <c r="E47" s="9" t="inlineStr">
+        <is>
+          <t>Rate 200</t>
+        </is>
+      </c>
       <c r="F47" s="8" t="inlineStr">
         <is>
           <t>ME</t>
@@ -1828,7 +1910,11 @@
           <t>UNB5005</t>
         </is>
       </c>
-      <c r="E48" s="9" t="inlineStr"/>
+      <c r="E48" s="9" t="inlineStr">
+        <is>
+          <t>Rate 200</t>
+        </is>
+      </c>
       <c r="F48" s="8" t="inlineStr">
         <is>
           <t>ME</t>
@@ -1852,7 +1938,11 @@
           <t>UNB5006</t>
         </is>
       </c>
-      <c r="E49" s="9" t="inlineStr"/>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>Rate 200</t>
+        </is>
+      </c>
       <c r="F49" s="8" t="inlineStr">
         <is>
           <t>ME</t>
@@ -2005,6 +2095,664 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D24"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Plan name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Rate ($/acct)</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Holdback %</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Rate 150</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="n">
+        <v>150</v>
+      </c>
+      <c r="C2" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Rate 175</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="n">
+        <v>175</v>
+      </c>
+      <c r="C3" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Rate 200</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>200</v>
+      </c>
+      <c r="C4" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Rate 210</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="n">
+        <v>210</v>
+      </c>
+      <c r="C5" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Rate 225</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>225</v>
+      </c>
+      <c r="C6" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Rate 240</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="n">
+        <v>240</v>
+      </c>
+      <c r="C7" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>Rate 250</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>250</v>
+      </c>
+      <c r="C8" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Rate 265</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>265</v>
+      </c>
+      <c r="C9" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>Rate 275</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="n">
+        <v>275</v>
+      </c>
+      <c r="C10" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="8" t="inlineStr">
+        <is>
+          <t>Rate 280</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>280</v>
+      </c>
+      <c r="C11" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Rate 290</t>
+        </is>
+      </c>
+      <c r="B12" s="8" t="n">
+        <v>290</v>
+      </c>
+      <c r="C12" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr">
+        <is>
+          <t>Rate 300</t>
+        </is>
+      </c>
+      <c r="B13" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="C13" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D13" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="8" t="inlineStr">
+        <is>
+          <t>Rate 300 AW</t>
+        </is>
+      </c>
+      <c r="B14" s="8" t="n">
+        <v>300</v>
+      </c>
+      <c r="C14" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="8" t="inlineStr">
+        <is>
+          <t>Rate 325</t>
+        </is>
+      </c>
+      <c r="B15" s="8" t="n">
+        <v>325</v>
+      </c>
+      <c r="C15" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D15" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="8" t="inlineStr">
+        <is>
+          <t>Rate 350</t>
+        </is>
+      </c>
+      <c r="B16" s="8" t="n">
+        <v>350</v>
+      </c>
+      <c r="C16" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D16" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="8" t="inlineStr">
+        <is>
+          <t>Rate 375</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n">
+        <v>375</v>
+      </c>
+      <c r="C17" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D17" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="8" t="inlineStr">
+        <is>
+          <t>400 Sub</t>
+        </is>
+      </c>
+      <c r="B18" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="C18" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="8" t="inlineStr">
+        <is>
+          <t>400 - Sub Dealer</t>
+        </is>
+      </c>
+      <c r="B19" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="C19" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D19" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="8" t="inlineStr">
+        <is>
+          <t>400 - Sub Dealer No Holdback</t>
+        </is>
+      </c>
+      <c r="B20" s="8" t="n">
+        <v>400</v>
+      </c>
+      <c r="C20" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Sub Dealer</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="inlineStr"/>
+      <c r="C21" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D21" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="8" t="inlineStr">
+        <is>
+          <t>Landon's Comp Plan</t>
+        </is>
+      </c>
+      <c r="B22" s="8" t="inlineStr"/>
+      <c r="C22" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="8" t="inlineStr">
+        <is>
+          <t>Enlite Plan</t>
+        </is>
+      </c>
+      <c r="B23" s="8" t="inlineStr"/>
+      <c r="C23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="8" t="inlineStr">
+        <is>
+          <t>Top G Plan</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="inlineStr"/>
+      <c r="C24" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>ISP name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Abbr</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+      <c r="D1" s="7" t="inlineStr">
+        <is>
+          <t>Rep-ID column on report</t>
+        </is>
+      </c>
+      <c r="E1" s="7" t="inlineStr">
+        <is>
+          <t>Has order #?</t>
+        </is>
+      </c>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Phone bonus $</t>
+        </is>
+      </c>
+      <c r="G1" s="7" t="inlineStr">
+        <is>
+          <t>Mesh bonus $</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Gonetspeed</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>GNS</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr"/>
+      <c r="E2" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F2" s="9" t="inlineStr"/>
+      <c r="G2" s="9" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>Brightspeed</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>BS</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr"/>
+      <c r="E3" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F3" s="9" t="inlineStr"/>
+      <c r="G3" s="9" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Joink / CTI</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>CTI</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr"/>
+      <c r="E4" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F4" s="9" t="inlineStr"/>
+      <c r="G4" s="9" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Fiber First</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>FF</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D5" s="9" t="inlineStr"/>
+      <c r="E5" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F5" s="9" t="inlineStr"/>
+      <c r="G5" s="9" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Lightcurve</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>LC</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr"/>
+      <c r="E6" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F6" s="9" t="inlineStr"/>
+      <c r="G6" s="9" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>Fatbeam</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>FB</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="D7" s="9" t="inlineStr"/>
+      <c r="E7" s="9" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+      <c r="F7" s="9" t="inlineStr"/>
+      <c r="G7" s="9" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2030,85 +2778,85 @@
     <col width="40" customWidth="1" min="15" max="15"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="10" t="inlineStr">
+    <row r="1" ht="24" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>Received</t>
         </is>
       </c>
-      <c r="B1" s="10" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Submitted by</t>
         </is>
       </c>
-      <c r="C1" s="10" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" s="10" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Blitz</t>
         </is>
       </c>
-      <c r="E1" s="10" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="F1" s="10" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="G1" s="10" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="H1" s="10" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>ISP(s)</t>
         </is>
       </c>
-      <c r="I1" s="10" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t># Reps</t>
         </is>
       </c>
-      <c r="J1" s="10" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Reps (name / ID / comp / change)</t>
         </is>
       </c>
-      <c r="K1" s="10" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Manager overrides</t>
         </is>
       </c>
-      <c r="L1" s="10" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Divisional overrides</t>
         </is>
       </c>
-      <c r="M1" s="10" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>New ISPs</t>
         </is>
       </c>
-      <c r="N1" s="10" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="O1" s="10" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Full summary</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>↑ Auto-filled by the intake form — one row per blitz. Do not edit the header row.</t>
         </is>

</xml_diff>

<commit_message>
Rename Roster "Region" column to "Office"
- Template: Office is now a yellow fill-in column; instructions reworded.
- Code.gs: ROSTER_HEADERS and readRoster field renamed region -> office.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/Unbreakable-Blitz-Intake-Template.xlsx
+++ b/template/Unbreakable-Blitz-Intake-Template.xlsx
@@ -500,13 +500,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:B21"/>
+  <dimension ref="B1:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="104" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -521,6 +522,7 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -531,7 +533,7 @@
     <row r="6">
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>• Roster — master rep list. The form's rep picker reads this. Fill the yellow Email column; verify Default plan.</t>
+          <t>• Roster — master rep list. The form's rep picker reads this. Fill the yellow Email + Office columns; verify Default plan.</t>
         </is>
       </c>
     </row>
@@ -549,6 +551,7 @@
         </is>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -570,6 +573,7 @@
         </is>
       </c>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -612,6 +616,7 @@
         </is>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -667,9 +672,9 @@
           <t>Default plan</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
-        <is>
-          <t>Region</t>
+      <c r="F1" s="7" t="inlineStr">
+        <is>
+          <t>Office</t>
         </is>
       </c>
     </row>
@@ -695,7 +700,7 @@
           <t>Rate 325</t>
         </is>
       </c>
-      <c r="F2" s="8" t="inlineStr">
+      <c r="F2" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -723,7 +728,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="F3" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -751,7 +756,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F4" s="8" t="inlineStr">
+      <c r="F4" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -783,7 +788,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F5" s="8" t="inlineStr">
+      <c r="F5" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -811,7 +816,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F6" s="8" t="inlineStr">
+      <c r="F6" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -835,7 +840,7 @@
         </is>
       </c>
       <c r="E7" s="9" t="inlineStr"/>
-      <c r="F7" s="8" t="inlineStr">
+      <c r="F7" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -863,7 +868,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F8" s="8" t="inlineStr">
+      <c r="F8" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -891,7 +896,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F9" s="8" t="inlineStr">
+      <c r="F9" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -919,7 +924,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F10" s="8" t="inlineStr">
+      <c r="F10" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -943,7 +948,7 @@
         </is>
       </c>
       <c r="E11" s="9" t="inlineStr"/>
-      <c r="F11" s="8" t="inlineStr">
+      <c r="F11" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -971,7 +976,7 @@
           <t>Rate 275</t>
         </is>
       </c>
-      <c r="F12" s="8" t="inlineStr">
+      <c r="F12" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -1003,7 +1008,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F13" s="8" t="inlineStr">
+      <c r="F13" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -1035,7 +1040,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F14" s="8" t="inlineStr">
+      <c r="F14" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -1067,7 +1072,7 @@
           <t>Rate 200</t>
         </is>
       </c>
-      <c r="F15" s="8" t="inlineStr">
+      <c r="F15" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -1091,7 +1096,7 @@
         </is>
       </c>
       <c r="E16" s="9" t="inlineStr"/>
-      <c r="F16" s="8" t="inlineStr">
+      <c r="F16" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -1119,7 +1124,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F17" s="8" t="inlineStr">
+      <c r="F17" s="9" t="inlineStr">
         <is>
           <t>NY</t>
         </is>
@@ -1143,7 +1148,7 @@
         </is>
       </c>
       <c r="E18" s="9" t="inlineStr"/>
-      <c r="F18" s="8" t="inlineStr">
+      <c r="F18" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1167,7 +1172,7 @@
         </is>
       </c>
       <c r="E19" s="9" t="inlineStr"/>
-      <c r="F19" s="8" t="inlineStr">
+      <c r="F19" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1195,7 +1200,7 @@
           <t>Rate 225</t>
         </is>
       </c>
-      <c r="F20" s="8" t="inlineStr">
+      <c r="F20" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1219,7 +1224,7 @@
         </is>
       </c>
       <c r="E21" s="9" t="inlineStr"/>
-      <c r="F21" s="8" t="inlineStr">
+      <c r="F21" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1247,7 +1252,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F22" s="8" t="inlineStr">
+      <c r="F22" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1275,7 +1280,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F23" s="8" t="inlineStr">
+      <c r="F23" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1303,7 +1308,7 @@
           <t>Rate 200</t>
         </is>
       </c>
-      <c r="F24" s="8" t="inlineStr">
+      <c r="F24" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1327,7 +1332,7 @@
         </is>
       </c>
       <c r="E25" s="9" t="inlineStr"/>
-      <c r="F25" s="8" t="inlineStr">
+      <c r="F25" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1351,7 +1356,7 @@
         </is>
       </c>
       <c r="E26" s="9" t="inlineStr"/>
-      <c r="F26" s="8" t="inlineStr">
+      <c r="F26" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1375,7 +1380,7 @@
         </is>
       </c>
       <c r="E27" s="9" t="inlineStr"/>
-      <c r="F27" s="8" t="inlineStr">
+      <c r="F27" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1399,7 +1404,7 @@
         </is>
       </c>
       <c r="E28" s="9" t="inlineStr"/>
-      <c r="F28" s="8" t="inlineStr">
+      <c r="F28" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1423,7 +1428,7 @@
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr"/>
-      <c r="F29" s="8" t="inlineStr">
+      <c r="F29" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1443,7 +1448,7 @@
         </is>
       </c>
       <c r="E30" s="9" t="inlineStr"/>
-      <c r="F30" s="8" t="inlineStr">
+      <c r="F30" s="9" t="inlineStr">
         <is>
           <t>MA</t>
         </is>
@@ -1471,7 +1476,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F31" s="8" t="inlineStr">
+      <c r="F31" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1495,7 +1500,7 @@
         </is>
       </c>
       <c r="E32" s="9" t="inlineStr"/>
-      <c r="F32" s="8" t="inlineStr">
+      <c r="F32" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1519,7 +1524,7 @@
         </is>
       </c>
       <c r="E33" s="9" t="inlineStr"/>
-      <c r="F33" s="8" t="inlineStr">
+      <c r="F33" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1543,7 +1548,7 @@
         </is>
       </c>
       <c r="E34" s="9" t="inlineStr"/>
-      <c r="F34" s="8" t="inlineStr">
+      <c r="F34" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1567,7 +1572,7 @@
         </is>
       </c>
       <c r="E35" s="9" t="inlineStr"/>
-      <c r="F35" s="8" t="inlineStr">
+      <c r="F35" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1595,7 +1600,7 @@
           <t>Rate 225</t>
         </is>
       </c>
-      <c r="F36" s="8" t="inlineStr">
+      <c r="F36" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1615,7 +1620,7 @@
         </is>
       </c>
       <c r="E37" s="9" t="inlineStr"/>
-      <c r="F37" s="8" t="inlineStr">
+      <c r="F37" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1643,7 +1648,7 @@
           <t>Rate 300</t>
         </is>
       </c>
-      <c r="F38" s="8" t="inlineStr">
+      <c r="F38" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1671,7 +1676,7 @@
           <t>Rate 225</t>
         </is>
       </c>
-      <c r="F39" s="8" t="inlineStr">
+      <c r="F39" s="9" t="inlineStr">
         <is>
           <t>AL</t>
         </is>
@@ -1695,7 +1700,7 @@
         </is>
       </c>
       <c r="E40" s="9" t="inlineStr"/>
-      <c r="F40" s="8" t="inlineStr">
+      <c r="F40" s="9" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
@@ -1719,7 +1724,7 @@
         </is>
       </c>
       <c r="E41" s="9" t="inlineStr"/>
-      <c r="F41" s="8" t="inlineStr">
+      <c r="F41" s="9" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
@@ -1747,7 +1752,7 @@
           <t>Rate 325</t>
         </is>
       </c>
-      <c r="F42" s="8" t="inlineStr">
+      <c r="F42" s="9" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
@@ -1775,7 +1780,7 @@
           <t>Rate 325</t>
         </is>
       </c>
-      <c r="F43" s="8" t="inlineStr">
+      <c r="F43" s="9" t="inlineStr">
         <is>
           <t>CT</t>
         </is>
@@ -1803,7 +1808,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F44" s="8" t="inlineStr">
+      <c r="F44" s="9" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
@@ -1831,7 +1836,7 @@
           <t>Rate 250</t>
         </is>
       </c>
-      <c r="F45" s="8" t="inlineStr">
+      <c r="F45" s="9" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
@@ -1859,7 +1864,7 @@
           <t>Rate 200</t>
         </is>
       </c>
-      <c r="F46" s="8" t="inlineStr">
+      <c r="F46" s="9" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
@@ -1887,7 +1892,7 @@
           <t>Rate 200</t>
         </is>
       </c>
-      <c r="F47" s="8" t="inlineStr">
+      <c r="F47" s="9" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
@@ -1915,7 +1920,7 @@
           <t>Rate 200</t>
         </is>
       </c>
-      <c r="F48" s="8" t="inlineStr">
+      <c r="F48" s="9" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
@@ -1943,7 +1948,7 @@
           <t>Rate 200</t>
         </is>
       </c>
-      <c r="F49" s="8" t="inlineStr">
+      <c r="F49" s="9" t="inlineStr">
         <is>
           <t>ME</t>
         </is>
@@ -1967,7 +1972,7 @@
         </is>
       </c>
       <c r="E50" s="9" t="inlineStr"/>
-      <c r="F50" s="8" t="inlineStr">
+      <c r="F50" s="9" t="inlineStr">
         <is>
           <t>Call Center</t>
         </is>
@@ -1991,7 +1996,7 @@
         </is>
       </c>
       <c r="E51" s="9" t="inlineStr"/>
-      <c r="F51" s="8" t="inlineStr">
+      <c r="F51" s="9" t="inlineStr">
         <is>
           <t>Call Center</t>
         </is>
@@ -2015,7 +2020,7 @@
         </is>
       </c>
       <c r="E52" s="9" t="inlineStr"/>
-      <c r="F52" s="8" t="inlineStr">
+      <c r="F52" s="9" t="inlineStr">
         <is>
           <t>Call Center</t>
         </is>
@@ -2039,7 +2044,7 @@
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr"/>
-      <c r="F53" s="8" t="inlineStr">
+      <c r="F53" s="9" t="inlineStr">
         <is>
           <t>Call Center</t>
         </is>
@@ -2063,7 +2068,7 @@
         </is>
       </c>
       <c r="E54" s="9" t="inlineStr"/>
-      <c r="F54" s="8" t="inlineStr">
+      <c r="F54" s="9" t="inlineStr">
         <is>
           <t>Call Center</t>
         </is>
@@ -2083,7 +2088,7 @@
         </is>
       </c>
       <c r="E55" s="9" t="inlineStr"/>
-      <c r="F55" s="8" t="inlineStr">
+      <c r="F55" s="9" t="inlineStr">
         <is>
           <t>Call Center</t>
         </is>

</xml_diff>

<commit_message>
Add Submission ID + per-rep "Rep detail" tab
- Each submission gets a unique ID (UNB-YYYYMMDD-NNN), computed under lock.
- New "Rep detail" tab: one row per rep per blitz with blitz context, plan,
  comp, new-rep flag, and the overrides resolved onto each rep (payroll-ready).
- Submissions tab gains the Submission ID as its first column.
- Template + setup menu updated to match.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/Unbreakable-Blitz-Intake-Template.xlsx
+++ b/template/Unbreakable-Blitz-Intake-Template.xlsx
@@ -12,6 +12,7 @@
     <sheet name="CompPlans" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="ISPs" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Submissions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Rep detail" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -500,14 +501,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:B21"/>
+  <dimension ref="B2:B21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
     <col width="104" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2">
       <c r="B2" s="1" t="inlineStr">
         <is>
@@ -522,7 +522,6 @@
         </is>
       </c>
     </row>
-    <row r="4"/>
     <row r="5">
       <c r="B5" s="3" t="inlineStr">
         <is>
@@ -551,7 +550,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="B10" s="3" t="inlineStr">
         <is>
@@ -573,7 +571,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="B14" s="3" t="inlineStr">
         <is>
@@ -616,7 +613,6 @@
         </is>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="B21" s="5" t="inlineStr">
         <is>
@@ -2763,98 +2759,104 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:Q2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="24" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="8" customWidth="1" min="9" max="9"/>
-    <col width="40" customWidth="1" min="10" max="10"/>
-    <col width="26" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="40" customWidth="1" min="11" max="11"/>
     <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="30" customWidth="1" min="13" max="13"/>
-    <col width="24" customWidth="1" min="14" max="14"/>
-    <col width="40" customWidth="1" min="15" max="15"/>
+    <col width="26" customWidth="1" min="13" max="13"/>
+    <col width="30" customWidth="1" min="14" max="14"/>
+    <col width="24" customWidth="1" min="15" max="15"/>
+    <col width="40" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
-    <row r="1" ht="24" customHeight="1">
+    <row r="1" ht="26" customHeight="1">
       <c r="A1" s="6" t="inlineStr">
         <is>
+          <t>Submission ID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
           <t>Received</t>
         </is>
       </c>
-      <c r="B1" s="6" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Submitted by</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Email</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Blitz</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>ISP(s)</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t># Reps</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Reps (name / ID / comp / change)</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Manager overrides</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>Divisional overrides</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>New ISPs</t>
         </is>
       </c>
-      <c r="N1" s="6" t="inlineStr">
+      <c r="O1" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
       </c>
-      <c r="O1" s="6" t="inlineStr">
+      <c r="P1" s="6" t="inlineStr">
         <is>
           <t>Full summary</t>
         </is>
@@ -2864,6 +2866,109 @@
       <c r="A2" s="10" t="inlineStr">
         <is>
           <t>↑ Auto-filled by the intake form — one row per blitz. Do not edit the header row.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:M2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="16" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Submission ID</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Received</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>Blitz</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>ISP(s)</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>Rep</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>UNB ID</t>
+        </is>
+      </c>
+      <c r="J1" s="6" t="inlineStr">
+        <is>
+          <t>Comp plan</t>
+        </is>
+      </c>
+      <c r="K1" s="6" t="inlineStr">
+        <is>
+          <t>Comp $</t>
+        </is>
+      </c>
+      <c r="L1" s="6" t="inlineStr">
+        <is>
+          <t>New rep?</t>
+        </is>
+      </c>
+      <c r="M1" s="6" t="inlineStr">
+        <is>
+          <t>Overrides on rep</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="10" t="inlineStr">
+        <is>
+          <t>↑ Auto-filled — one row per rep per blitz (payroll-friendly). Do not edit the header row.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add "add reps to existing blitz" mode + Offices/Blitzes tabs
- Form gains a mode toggle: New blitz | Add reps to existing.
- New blitz: Office dropdown (from Offices tab / Roster); blitz name composed
  as "Office · City ST"; new blitzes auto-register on the Blitzes tab.
- Add reps: pick an existing blitz (grouped by office) from the Blitzes tab;
  reps/overrides append to that blitz, inheriting its details + ISPs.
- Backend: doGet returns offices + blitzes; Rep detail gains an Office column;
  Submissions marks add-on rows "(+reps added)".
- Template: Offices + Blitzes tabs seeded with examples.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/Unbreakable-Blitz-Intake-Template.xlsx
+++ b/template/Unbreakable-Blitz-Intake-Template.xlsx
@@ -9,10 +9,12 @@
   <sheets>
     <sheet name="Instructions" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Roster" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="CompPlans" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="ISPs" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Submissions" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Rep detail" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Blitzes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Offices" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="CompPlans" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="ISPs" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Submissions" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Rep detail" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -2101,6 +2103,198 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:I3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Blitz name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="C1" s="6" t="inlineStr">
+        <is>
+          <t>City</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+      <c r="F1" s="6" t="inlineStr">
+        <is>
+          <t>End</t>
+        </is>
+      </c>
+      <c r="G1" s="6" t="inlineStr">
+        <is>
+          <t>Manager</t>
+        </is>
+      </c>
+      <c r="H1" s="6" t="inlineStr">
+        <is>
+          <t>ISP(s)</t>
+        </is>
+      </c>
+      <c r="I1" s="6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Utah Allwest · Geneva NY</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>Utah Allwest</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>Geneva</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>NY</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-05</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>2026-07-18</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Calijah Hunter</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Gonetspeed</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="10" t="inlineStr">
+        <is>
+          <t>↑ Example row — the form adds new blitzes here automatically; set Active to 'no' to hide one from the picker.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="6" t="inlineStr">
+        <is>
+          <t>Office name</t>
+        </is>
+      </c>
+      <c r="B1" s="6" t="inlineStr">
+        <is>
+          <t>Active</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>Utah Allwest</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>The GRIT</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>Isaac Maughn Group</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>yes</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -2543,7 +2737,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2753,13 +2947,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -2874,28 +3068,29 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M2"/>
+  <dimension ref="A1:O2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
-    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="24" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -2916,50 +3111,55 @@
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
+          <t>Office</t>
+        </is>
+      </c>
+      <c r="E1" s="6" t="inlineStr">
+        <is>
           <t>Start</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>End</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Manager</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>ISP(s)</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Rep</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>UNB ID</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Comp plan</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="L1" s="6" t="inlineStr">
         <is>
           <t>Comp $</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="M1" s="6" t="inlineStr">
         <is>
           <t>New rep?</t>
         </is>
       </c>
-      <c r="M1" s="6" t="inlineStr">
+      <c r="N1" s="6" t="inlineStr">
         <is>
           <t>Overrides on rep</t>
         </is>

</xml_diff>

<commit_message>
Add recurring + one-time recruiter override types
Override Type now offers Manager, Divisional, Recruiter — recurring, and
Recruiter — one-time. Backend tags recruiter overrides with their frequency in
both the Submissions override column and the per-rep Rep detail column; the
"Manager overrides" column is renamed "Manager / recruiter overrides".
No sheet rebuild needed (columns unchanged) — just redeploy Code.gs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/template/Unbreakable-Blitz-Intake-Template.xlsx
+++ b/template/Unbreakable-Blitz-Intake-Template.xlsx
@@ -3032,7 +3032,7 @@
       </c>
       <c r="L1" s="6" t="inlineStr">
         <is>
-          <t>Manager overrides</t>
+          <t>Manager / recruiter overrides</t>
         </is>
       </c>
       <c r="M1" s="6" t="inlineStr">
@@ -3074,7 +3074,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:N2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>

</xml_diff>